<commit_message>
Actualizar ingesta para almacenar detalles de películas
</commit_message>
<xml_diff>
--- a/tmdb_movies.xlsx
+++ b/tmdb_movies.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,7 +501,42 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>page</t>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>runtime</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>genres</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>production_companies</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>spoken_languages</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>homepage</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>tagline</t>
         </is>
       </c>
     </row>
@@ -538,7 +573,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>79.65900000000001</v>
+        <v>111.523</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -562,10 +597,41 @@
         <v>7.608</v>
       </c>
       <c r="N2" t="n">
-        <v>12292</v>
+        <v>12294</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>460000000</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2320250281</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>192</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>['Science Fiction', 'Adventure', 'Action']</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>['20th Century Studios', 'Lightstorm Entertainment']</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>https://www.avatar.com/movies/avatar-the-way-of-water</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Return to Pandora.</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -574,7 +640,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>/AeK2MPOpYrOOgZNfFnfwp0L8tNn.jpg</t>
+          <t>/zD5v1E4joAzFvmAEytt7fM3ivyT.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -601,7 +667,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>107.608</v>
+        <v>150.651</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -625,10 +691,41 @@
         <v>7.9</v>
       </c>
       <c r="N3" t="n">
-        <v>20547</v>
+        <v>20552</v>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>200000000</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1921847111</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>148</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>['Action', 'Adventure', 'Science Fiction']</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>['Marvel Studios', 'Pascal Pictures', 'Columbia Pictures']</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>['English', '']</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>https://www.sonypictures.com/movies/spidermannowayhome</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>The Multiverse unleashed.</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -664,7 +761,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>181.517</v>
+        <v>254.124</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -685,13 +782,44 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>7.56</v>
+        <v>7.6</v>
       </c>
       <c r="N4" t="n">
-        <v>5578</v>
+        <v>5581</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>200000000</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1698863816</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>97</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>['Animation', 'Adventure', 'Comedy', 'Family']</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>['Walt Disney Pictures', 'Pixar']</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>https://movies.disney.com/inside-out-2</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Make room for new emotions.</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -727,7 +855,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>104.978</v>
+        <v>146.969</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -748,13 +876,44 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>8.199999999999999</v>
+        <v>8.186</v>
       </c>
       <c r="N5" t="n">
-        <v>9601</v>
+        <v>9605</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>170000000</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1488732821</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>131</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>['Action', 'Drama']</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>['Skydance Media', 'Don Simpson/Jerry Bruckheimer Films', 'Paramount Pictures']</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>https://www.topgunmovie.com</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Feel the need... The need for speed.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -790,7 +949,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>62.15</v>
+        <v>87.01000000000001</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -814,10 +973,41 @@
         <v>6.984</v>
       </c>
       <c r="N6" t="n">
-        <v>9591</v>
+        <v>9597</v>
       </c>
       <c r="O6" t="n">
-        <v>1</v>
+        <v>145000000</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1445638421</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>114</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>['Comedy', 'Adventure']</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>['LuckyChap Entertainment', 'Heyday Films', 'NB/GG Pictures', 'Mattel', 'Warner Bros. Pictures']</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>https://www.barbie-themovie.com</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>She's everything. He's just Ken.</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -853,7 +1043,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>84.819</v>
+        <v>118.747</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -877,10 +1067,41 @@
         <v>7.632</v>
       </c>
       <c r="N7" t="n">
-        <v>9470</v>
+        <v>9473</v>
       </c>
       <c r="O7" t="n">
-        <v>1</v>
+        <v>100000000</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1362000000</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>93</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>['Animation', 'Family', 'Adventure', 'Fantasy', 'Comedy']</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>['Universal Pictures', 'Illumination', 'Nintendo']</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>https://www.uphe.com/movies/the-super-mario-bros-movie</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Not all heroes wear capes. Some wear overalls.</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -916,7 +1137,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>228.761</v>
+        <v>320.265</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -937,13 +1158,44 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>7.619</v>
+        <v>7.6</v>
       </c>
       <c r="N8" t="n">
-        <v>6776</v>
+        <v>6781</v>
       </c>
       <c r="O8" t="n">
-        <v>1</v>
+        <v>200000000</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1338073645</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>128</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>['Action', 'Comedy', 'Science Fiction']</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>['Marvel Studios', 'Maximum Effort', '21 Laps Entertainment', '20th Century Studios', 'Kevin Feige Productions', 'TSG Entertainment']</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>https://www.marvel.com/movies/deadpool-and-wolverine</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Come together.</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -979,7 +1231,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1361.081</v>
+        <v>1623.864</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1000,13 +1252,44 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>7.2</v>
+        <v>7.157</v>
       </c>
       <c r="N9" t="n">
-        <v>1703</v>
+        <v>1721</v>
       </c>
       <c r="O9" t="n">
-        <v>1</v>
+        <v>150000000</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1044396565</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>99</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>['Animation', 'Adventure', 'Family', 'Comedy']</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>['Walt Disney Pictures', 'Walt Disney Animation Studios', 'Walt Disney Animation Studios']</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>['English', 'Italiano']</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>https://movies.disney.com/moana-2</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>The ocean is calling them back.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1042,7 +1325,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>126.638</v>
+        <v>147.765</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1066,10 +1349,41 @@
         <v>6.7</v>
       </c>
       <c r="N10" t="n">
-        <v>6251</v>
+        <v>6255</v>
       </c>
       <c r="O10" t="n">
-        <v>1</v>
+        <v>165000000</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1001978080</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>147</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>['Adventure', 'Action', 'Science Fiction']</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>['Amblin Entertainment', 'Universal Pictures']</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>https://www.jurassicworld.com</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>The epic conclusion of the Jurassic era.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1105,7 +1419,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>209.01</v>
+        <v>292.614</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1126,13 +1440,44 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>7.1</v>
+        <v>7.061</v>
       </c>
       <c r="N11" t="n">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="O11" t="n">
-        <v>1</v>
+        <v>100000000</v>
+      </c>
+      <c r="P11" t="n">
+        <v>969280910</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>94</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>['Animation', 'Family', 'Comedy', 'Science Fiction']</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>['Universal Pictures', 'Illumination']</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>https://www.despicable.me</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>This daddy’s a baddie.</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1168,7 +1513,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>56.552</v>
+        <v>79.173</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1189,13 +1534,44 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>7.267</v>
+        <v>7.3</v>
       </c>
       <c r="N12" t="n">
         <v>9370</v>
       </c>
       <c r="O12" t="n">
-        <v>1</v>
+        <v>200000000</v>
+      </c>
+      <c r="P12" t="n">
+        <v>955775804</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>126</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>['Fantasy', 'Action', 'Adventure']</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>['Marvel Studios', 'Kevin Feige Productions']</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>['广州话 / 廣州話', 'English', 'Español']</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://www.marvel.com/movies/doctor-strange-in-the-multiverse-of-madness</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Enter a new dimension of Strange.</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1231,7 +1607,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>72.999</v>
+        <v>102.199</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1255,10 +1631,41 @@
         <v>8.1</v>
       </c>
       <c r="N13" t="n">
-        <v>9857</v>
+        <v>9867</v>
       </c>
       <c r="O13" t="n">
-        <v>1</v>
+        <v>100000000</v>
+      </c>
+      <c r="P13" t="n">
+        <v>952000000</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>181</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>['Drama', 'History']</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>['Syncopy', 'Universal Pictures', 'Atlas Entertainment', 'Breakheart Films', 'Peters Creek Entertainment']</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>['Nederlands', 'English']</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>https://www.universalpictures.com/movies/oppenheimer</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>The world forever changes.</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1294,7 +1701,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>35.589</v>
+        <v>49.825</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1315,13 +1722,44 @@
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>7.302</v>
+        <v>7.3</v>
       </c>
       <c r="N14" t="n">
         <v>3680</v>
       </c>
       <c r="O14" t="n">
-        <v>1</v>
+        <v>85000000</v>
+      </c>
+      <c r="P14" t="n">
+        <v>940203765</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>87</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>['Animation', 'Comedy', 'Family', 'Adventure']</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>['Universal Pictures', 'Illumination']</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>https://www.minionsmovie.com/</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>A villain will rise.</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1353,7 +1791,7 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>9.869999999999999</v>
+        <v>9.746</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1380,7 +1818,34 @@
         <v>105</v>
       </c>
       <c r="O15" t="n">
-        <v>1</v>
+        <v>200000000</v>
+      </c>
+      <c r="P15" t="n">
+        <v>902540935</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>178</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>['Drama', 'War']</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>['Bona Film Group', 'Shanghai Film Group', 'DF Pictures', 'Alibaba Pictures Group', 'China Film Group Corporation', 'Distribution Workshop', 'Huaxia Film Distribution', 'Just Creative Studio']</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>['普通话', 'English']</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Do they fall out of the goddamn sky?</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1416,7 +1881,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>58.598</v>
+        <v>82.03700000000001</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1440,10 +1905,41 @@
         <v>7.1</v>
       </c>
       <c r="N16" t="n">
-        <v>6684</v>
+        <v>6686</v>
       </c>
       <c r="O16" t="n">
-        <v>1</v>
+        <v>250000000</v>
+      </c>
+      <c r="P16" t="n">
+        <v>859102154</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>162</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>['Action', 'Adventure', 'Science Fiction']</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>['Marvel Studios']</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>['English', 'Français', '', 'Español', '']</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>https://wakandaforevertickets.com</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Forever.</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1479,7 +1975,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>63.091</v>
+        <v>88.327</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1503,10 +1999,41 @@
         <v>8</v>
       </c>
       <c r="N17" t="n">
-        <v>7159</v>
+        <v>7160</v>
       </c>
       <c r="O17" t="n">
-        <v>1</v>
+        <v>250000000</v>
+      </c>
+      <c r="P17" t="n">
+        <v>845600000</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>150</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>['Science Fiction', 'Adventure', 'Action']</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>['Marvel Studios', 'Kevin Feige Productions']</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>https://www.marvel.com/movies/guardians-of-the-galaxy-volume-3</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Once more with feeling.</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1538,7 +2065,7 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>6.964</v>
+        <v>8.307</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1565,8 +2092,31 @@
         <v>147</v>
       </c>
       <c r="O18" t="n">
-        <v>1</v>
-      </c>
+        <v>59000000</v>
+      </c>
+      <c r="P18" t="n">
+        <v>822049668</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>128</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>['Drama', 'Comedy', 'Fantasy']</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>['Alibaba Pictures Group', 'Tianjin Maoyan Media', 'Beijing Big Bowl Entertainment Culture Media', 'Beijing Culture', 'Beijing Cheering Times Culture &amp; Entertainment', 'Shanghai Ruyi Film &amp; TV Production']</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>['普通话']</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="b">
@@ -1601,7 +2151,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>29.744</v>
+        <v>41.642</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1622,13 +2172,44 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>7.368</v>
+        <v>7.4</v>
       </c>
       <c r="N19" t="n">
-        <v>6406</v>
+        <v>6407</v>
       </c>
       <c r="O19" t="n">
-        <v>1</v>
+        <v>250000000</v>
+      </c>
+      <c r="P19" t="n">
+        <v>774153024</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>163</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>['Action', 'Thriller', 'Adventure']</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>['EON Productions', 'Metro-Goldwyn-Mayer']</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>['Español', 'English', 'Italiano', 'Français', 'Pусский']</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>https://www.007.com/no-time-to-die/</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>The mission that changes everything begins…</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1664,7 +2245,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>55.633</v>
+        <v>77.886</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1688,10 +2269,41 @@
         <v>7.7</v>
       </c>
       <c r="N20" t="n">
-        <v>10663</v>
+        <v>10665</v>
       </c>
       <c r="O20" t="n">
-        <v>1</v>
+        <v>185000000</v>
+      </c>
+      <c r="P20" t="n">
+        <v>772319315</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>177</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>['Crime', 'Mystery', 'Thriller']</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>['6th &amp; Idaho Motion Picture Company', 'Dylan Clark Productions', 'DC Films', 'Warner Bros. Pictures']</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>https://www.thebatman.com</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Unmask the truth.</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1727,7 +2339,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>39.69</v>
+        <v>55.566</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1751,10 +2363,41 @@
         <v>6.422</v>
       </c>
       <c r="N21" t="n">
-        <v>7773</v>
+        <v>7775</v>
       </c>
       <c r="O21" t="n">
-        <v>1</v>
+        <v>250000000</v>
+      </c>
+      <c r="P21" t="n">
+        <v>760900000</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>119</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>['Fantasy', 'Action', 'Comedy']</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>['Marvel Studios', 'Kevin Feige Productions']</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>['English']</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>https://www.marvel.com/movies/thor-love-and-thunder</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>The one is not the only.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>